<commit_message>
Fix lookup keys containing '~' (Excel wildcard escape) so asphalt layer units resolve
Claude-Session: https://claude.ai/code/session_01RwMurm2uiMMwxjQxmRaq3G
</commit_message>
<xml_diff>
--- a/공기산정_2026기준.xlsx
+++ b/공기산정_2026기준.xlsx
@@ -90939,7 +90939,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5-7㎝)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -90959,7 +90959,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 8~10㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 8-10㎝)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -90979,7 +90979,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5-7㎝)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -92300,7 +92300,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5-7㎝)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -92332,7 +92332,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5-7㎝)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -92403,7 +92403,7 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5-7㎝)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -92415,7 +92415,7 @@
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5~7㎝)</t>
+          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5-7㎝)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">

</xml_diff>

<commit_message>
Add category filter for the work-item dropdown
Claude-Session: https://claude.ai/code/session_01RwMurm2uiMMwxjQxmRaq3G
</commit_message>
<xml_diff>
--- a/공기산정_2026기준.xlsx
+++ b/공기산정_2026기준.xlsx
@@ -4461,6 +4461,23 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="131" t="inlineStr">
+        <is>
+          <t>공종 목록 분류 (선택 범위 좁히기)</t>
+        </is>
+      </c>
+      <c r="B26" s="139" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>※ 분류를 고르면 아래 공종 칸의 목록이 그 분류의 공종만 보입니다.</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" s="131" t="inlineStr">
         <is>
@@ -8212,7 +8229,7 @@
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=공종프리셋!$A$1:$F$1</formula1>
     </dataValidation>
@@ -8225,8 +8242,11 @@
     <dataValidation sqref="E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
+    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>='1일작업량(토목)'!$F$2:$F$9</formula1>
+    </dataValidation>
     <dataValidation sqref="A29 A30 A31 A32 A33 A34 A35 A36 A37 A38 A39 A40 A41 A42 A43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='1일작업량(토목)'!$A$2:$A$115</formula1>
+      <formula1>=OFFSET('1일작업량(토목)'!$A$1,INDEX('1일작업량(토목)'!$G$2:$G$9,MATCH($B$26,'1일작업량(토목)'!$F$2:$F$9,0)),0,INDEX('1일작업량(토목)'!$H$2:$H$9,MATCH($B$26,'1일작업량(토목)'!$F$2:$F$9,0)),1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -89766,12 +89786,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" style="92" min="1" max="1"/>
     <col width="20" customWidth="1" style="92" min="3" max="3"/>
     <col width="22" customWidth="1" style="92" min="4" max="4"/>
+    <col width="16" customWidth="1" style="92" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -89795,6 +89816,21 @@
           <t>원문 표기 (부록 4)</t>
         </is>
       </c>
+      <c r="F1" s="134" t="inlineStr">
+        <is>
+          <t>분류 필터</t>
+        </is>
+      </c>
+      <c r="G1" s="134" t="inlineStr">
+        <is>
+          <t>시작 위치</t>
+        </is>
+      </c>
+      <c r="H1" s="134" t="inlineStr">
+        <is>
+          <t>개수</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -89815,6 +89851,17 @@
           <t>77일/개소</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>114</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -89835,6 +89882,17 @@
           <t>30m/일</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>공통가설공사</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -89855,6 +89913,17 @@
           <t>30m/일</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>토공사</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -89875,6 +89944,17 @@
           <t>82㎥/일</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>배수공사</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>36</v>
+      </c>
+      <c r="H5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -89895,6 +89975,17 @@
           <t>102㎡/일</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>포장공사</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>48</v>
+      </c>
+      <c r="H6" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -89915,6 +90006,17 @@
           <t>8본/일</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>교량공사</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>74</v>
+      </c>
+      <c r="H7" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -89935,6 +90037,17 @@
           <t>10본/일</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>터널공사</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>86</v>
+      </c>
+      <c r="H8" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -89954,6 +90067,17 @@
         <is>
           <t>6본/일</t>
         </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>부대공사</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>103</v>
+      </c>
+      <c r="H9" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Use named ranges + INDIRECT for the category-filtered work-item dropdown
Claude-Session: https://claude.ai/code/session_01RwMurm2uiMMwxjQxmRaq3G
</commit_message>
<xml_diff>
--- a/공기산정_2026기준.xlsx
+++ b/공기산정_2026기준.xlsx
@@ -21,6 +21,14 @@
     <definedName name="내선전공">#REF!</definedName>
     <definedName name="보통인부">#REF!</definedName>
     <definedName name="프랜트전공">#REF!</definedName>
+    <definedName name="전체">'1일작업량(토목)'!$A$2:$A$115</definedName>
+    <definedName name="공통가설공사">'1일작업량(토목)'!$A$2:$A$11</definedName>
+    <definedName name="토공사">'1일작업량(토목)'!$A$12:$A$36</definedName>
+    <definedName name="배수공사">'1일작업량(토목)'!$A$37:$A$48</definedName>
+    <definedName name="포장공사">'1일작업량(토목)'!$A$49:$A$74</definedName>
+    <definedName name="교량공사">'1일작업량(토목)'!$A$75:$A$86</definedName>
+    <definedName name="터널공사">'1일작업량(토목)'!$A$87:$A$103</definedName>
+    <definedName name="부대공사">'1일작업량(토목)'!$A$104:$A$115</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'공기산정'!$A$1:$V$39</definedName>
   </definedNames>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
@@ -8246,7 +8254,7 @@
       <formula1>='1일작업량(토목)'!$F$2:$F$9</formula1>
     </dataValidation>
     <dataValidation sqref="A29 A30 A31 A32 A33 A34 A35 A36 A37 A38 A39 A40 A41 A42 A43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=OFFSET('1일작업량(토목)'!$A$1,INDEX('1일작업량(토목)'!$G$2:$G$9,MATCH($B$26,'1일작업량(토목)'!$F$2:$F$9,0)),0,INDEX('1일작업량(토목)'!$H$2:$H$9,MATCH($B$26,'1일작업량(토목)'!$F$2:$F$9,0)),1)</formula1>
+      <formula1>=INDIRECT($B$26)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Make work-item dropdown source a static range filled by formulas (works in Hancom/Google Sheets/mobile)
Claude-Session: https://claude.ai/code/session_01RwMurm2uiMMwxjQxmRaq3G
</commit_message>
<xml_diff>
--- a/공기산정_2026기준.xlsx
+++ b/공기산정_2026기준.xlsx
@@ -21,14 +21,6 @@
     <definedName name="내선전공">#REF!</definedName>
     <definedName name="보통인부">#REF!</definedName>
     <definedName name="프랜트전공">#REF!</definedName>
-    <definedName name="전체">'1일작업량(토목)'!$A$2:$A$115</definedName>
-    <definedName name="공통가설공사">'1일작업량(토목)'!$A$2:$A$11</definedName>
-    <definedName name="토공사">'1일작업량(토목)'!$A$12:$A$36</definedName>
-    <definedName name="배수공사">'1일작업량(토목)'!$A$37:$A$48</definedName>
-    <definedName name="포장공사">'1일작업량(토목)'!$A$49:$A$74</definedName>
-    <definedName name="교량공사">'1일작업량(토목)'!$A$75:$A$86</definedName>
-    <definedName name="터널공사">'1일작업량(토목)'!$A$87:$A$103</definedName>
-    <definedName name="부대공사">'1일작업량(토목)'!$A$104:$A$115</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'공기산정'!$A$1:$V$39</definedName>
   </definedNames>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
@@ -8254,7 +8246,7 @@
       <formula1>='1일작업량(토목)'!$F$2:$F$9</formula1>
     </dataValidation>
     <dataValidation sqref="A29 A30 A31 A32 A33 A34 A35 A36 A37 A38 A39 A40 A41 A42 A43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT($B$26)</formula1>
+      <formula1>='1일작업량(토목)'!$J$2:$J$115</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -89794,13 +89786,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" style="92" min="1" max="1"/>
     <col width="20" customWidth="1" style="92" min="3" max="3"/>
     <col width="22" customWidth="1" style="92" min="4" max="4"/>
     <col width="16" customWidth="1" style="92" min="6" max="6"/>
+    <col width="70" customWidth="1" style="92" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -89839,6 +89832,11 @@
           <t>개수</t>
         </is>
       </c>
+      <c r="J1" s="134" t="inlineStr">
+        <is>
+          <t>필터된 공종 목록 (자동, 공종 칸 드롭다운의 원본)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -89870,6 +89868,10 @@
       <c r="H2" t="n">
         <v>114</v>
       </c>
+      <c r="J2">
+        <f>IF(ROWS($J$2:J2)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J2)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -89901,6 +89903,10 @@
       <c r="H3" t="n">
         <v>10</v>
       </c>
+      <c r="J3">
+        <f>IF(ROWS($J$2:J3)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J3)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -89932,6 +89938,10 @@
       <c r="H4" t="n">
         <v>25</v>
       </c>
+      <c r="J4">
+        <f>IF(ROWS($J$2:J4)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J4)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -89963,6 +89973,10 @@
       <c r="H5" t="n">
         <v>12</v>
       </c>
+      <c r="J5">
+        <f>IF(ROWS($J$2:J5)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J5)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -89994,6 +90008,10 @@
       <c r="H6" t="n">
         <v>26</v>
       </c>
+      <c r="J6">
+        <f>IF(ROWS($J$2:J6)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J6)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -90025,6 +90043,10 @@
       <c r="H7" t="n">
         <v>12</v>
       </c>
+      <c r="J7">
+        <f>IF(ROWS($J$2:J7)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J7)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -90056,6 +90078,10 @@
       <c r="H8" t="n">
         <v>17</v>
       </c>
+      <c r="J8">
+        <f>IF(ROWS($J$2:J8)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J8)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -90087,6 +90113,10 @@
       <c r="H9" t="n">
         <v>12</v>
       </c>
+      <c r="J9">
+        <f>IF(ROWS($J$2:J9)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J9)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -90107,6 +90137,10 @@
           <t>8본/일</t>
         </is>
       </c>
+      <c r="J10">
+        <f>IF(ROWS($J$2:J10)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J10)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -90127,6 +90161,10 @@
           <t>8본/일</t>
         </is>
       </c>
+      <c r="J11">
+        <f>IF(ROWS($J$2:J11)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J11)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -90147,6 +90185,10 @@
           <t>54㎥/일</t>
         </is>
       </c>
+      <c r="J12">
+        <f>IF(ROWS($J$2:J12)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J12)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -90167,6 +90209,10 @@
           <t>1,375㎡/일</t>
         </is>
       </c>
+      <c r="J13">
+        <f>IF(ROWS($J$2:J13)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J13)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -90187,6 +90233,10 @@
           <t>1,110㎡/일</t>
         </is>
       </c>
+      <c r="J14">
+        <f>IF(ROWS($J$2:J14)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J14)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -90207,6 +90257,10 @@
           <t>1,915㎡/일</t>
         </is>
       </c>
+      <c r="J15">
+        <f>IF(ROWS($J$2:J15)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J15)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -90227,6 +90281,10 @@
           <t>520㎥/일</t>
         </is>
       </c>
+      <c r="J16">
+        <f>IF(ROWS($J$2:J16)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J16)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -90247,6 +90305,10 @@
           <t>367㎥/일</t>
         </is>
       </c>
+      <c r="J17">
+        <f>IF(ROWS($J$2:J17)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J17)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -90267,6 +90329,10 @@
           <t>27㎥/일</t>
         </is>
       </c>
+      <c r="J18">
+        <f>IF(ROWS($J$2:J18)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J18)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -90287,6 +90353,10 @@
           <t>83㎥/일</t>
         </is>
       </c>
+      <c r="J19">
+        <f>IF(ROWS($J$2:J19)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J19)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -90307,6 +90377,10 @@
           <t>349㎥/일</t>
         </is>
       </c>
+      <c r="J20">
+        <f>IF(ROWS($J$2:J20)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J20)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -90327,6 +90401,10 @@
           <t>25㎥/일</t>
         </is>
       </c>
+      <c r="J21">
+        <f>IF(ROWS($J$2:J21)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J21)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -90347,6 +90425,10 @@
           <t>18㎥/일</t>
         </is>
       </c>
+      <c r="J22">
+        <f>IF(ROWS($J$2:J22)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J22)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -90367,6 +90449,10 @@
           <t>745㎥/일</t>
         </is>
       </c>
+      <c r="J23">
+        <f>IF(ROWS($J$2:J23)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J23)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -90387,6 +90473,10 @@
           <t>1,118㎥/일</t>
         </is>
       </c>
+      <c r="J24">
+        <f>IF(ROWS($J$2:J24)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J24)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -90407,6 +90497,10 @@
           <t>647㎥/일</t>
         </is>
       </c>
+      <c r="J25">
+        <f>IF(ROWS($J$2:J25)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J25)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -90427,6 +90521,10 @@
           <t>1,231㎥/일</t>
         </is>
       </c>
+      <c r="J26">
+        <f>IF(ROWS($J$2:J26)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J26)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -90447,6 +90545,10 @@
           <t>42㎥/일</t>
         </is>
       </c>
+      <c r="J27">
+        <f>IF(ROWS($J$2:J27)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J27)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -90467,6 +90569,10 @@
           <t>3,571㎡/일</t>
         </is>
       </c>
+      <c r="J28">
+        <f>IF(ROWS($J$2:J28)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J28)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -90487,6 +90593,10 @@
           <t>421㎥/일</t>
         </is>
       </c>
+      <c r="J29">
+        <f>IF(ROWS($J$2:J29)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J29)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -90507,6 +90617,10 @@
           <t>9,396m/일</t>
         </is>
       </c>
+      <c r="J30">
+        <f>IF(ROWS($J$2:J30)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J30)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -90527,6 +90641,10 @@
           <t>1,597㎥/일</t>
         </is>
       </c>
+      <c r="J31">
+        <f>IF(ROWS($J$2:J31)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J31)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -90547,6 +90665,10 @@
           <t>383㎥/일</t>
         </is>
       </c>
+      <c r="J32">
+        <f>IF(ROWS($J$2:J32)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J32)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -90567,6 +90689,10 @@
           <t>14본/일</t>
         </is>
       </c>
+      <c r="J33">
+        <f>IF(ROWS($J$2:J33)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J33)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -90587,6 +90713,10 @@
           <t>2.2본/일</t>
         </is>
       </c>
+      <c r="J34">
+        <f>IF(ROWS($J$2:J34)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J34)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -90607,6 +90737,10 @@
           <t>505㎡/일</t>
         </is>
       </c>
+      <c r="J35">
+        <f>IF(ROWS($J$2:J35)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J35)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -90627,6 +90761,10 @@
           <t>64m/일</t>
         </is>
       </c>
+      <c r="J36">
+        <f>IF(ROWS($J$2:J36)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J36)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -90647,6 +90785,10 @@
           <t>42일/15m/1span</t>
         </is>
       </c>
+      <c r="J37">
+        <f>IF(ROWS($J$2:J37)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J37)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -90667,6 +90809,10 @@
           <t>27일/15m/1span</t>
         </is>
       </c>
+      <c r="J38">
+        <f>IF(ROWS($J$2:J38)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J38)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -90687,6 +90833,10 @@
           <t>13일/개소</t>
         </is>
       </c>
+      <c r="J39">
+        <f>IF(ROWS($J$2:J39)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J39)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -90707,6 +90857,10 @@
           <t>43m/일</t>
         </is>
       </c>
+      <c r="J40">
+        <f>IF(ROWS($J$2:J40)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J40)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -90727,6 +90881,10 @@
           <t>38m/일</t>
         </is>
       </c>
+      <c r="J41">
+        <f>IF(ROWS($J$2:J41)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J41)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -90747,6 +90905,10 @@
           <t>3m/일</t>
         </is>
       </c>
+      <c r="J42">
+        <f>IF(ROWS($J$2:J42)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J42)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -90767,6 +90929,10 @@
           <t>25일/15m/1span</t>
         </is>
       </c>
+      <c r="J43">
+        <f>IF(ROWS($J$2:J43)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J43)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -90787,6 +90953,10 @@
           <t>14㎡/일</t>
         </is>
       </c>
+      <c r="J44">
+        <f>IF(ROWS($J$2:J44)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J44)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -90807,6 +90977,10 @@
           <t>8일/20m/1span</t>
         </is>
       </c>
+      <c r="J45">
+        <f>IF(ROWS($J$2:J45)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J45)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -90827,6 +91001,10 @@
           <t>9일/20m/1span</t>
         </is>
       </c>
+      <c r="J46">
+        <f>IF(ROWS($J$2:J46)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J46)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -90847,6 +91025,10 @@
           <t>8일/20m/1span</t>
         </is>
       </c>
+      <c r="J47">
+        <f>IF(ROWS($J$2:J47)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J47)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -90867,6 +91049,10 @@
           <t>8일/20m/1span</t>
         </is>
       </c>
+      <c r="J48">
+        <f>IF(ROWS($J$2:J48)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J48)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -90887,6 +91073,10 @@
           <t>1,900m/일</t>
         </is>
       </c>
+      <c r="J49">
+        <f>IF(ROWS($J$2:J49)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J49)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -90907,6 +91097,10 @@
           <t>1,600m/일</t>
         </is>
       </c>
+      <c r="J50">
+        <f>IF(ROWS($J$2:J50)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J50)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -90927,6 +91121,10 @@
           <t>5일</t>
         </is>
       </c>
+      <c r="J51">
+        <f>IF(ROWS($J$2:J51)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J51)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -90947,6 +91145,10 @@
           <t>600㎥/일</t>
         </is>
       </c>
+      <c r="J52">
+        <f>IF(ROWS($J$2:J52)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J52)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -90967,6 +91169,10 @@
           <t>550㎥/일</t>
         </is>
       </c>
+      <c r="J53">
+        <f>IF(ROWS($J$2:J53)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J53)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -90987,6 +91193,10 @@
           <t>1,900m/일</t>
         </is>
       </c>
+      <c r="J54">
+        <f>IF(ROWS($J$2:J54)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J54)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -91007,6 +91217,10 @@
           <t>1,600m/일</t>
         </is>
       </c>
+      <c r="J55">
+        <f>IF(ROWS($J$2:J55)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J55)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -91027,6 +91241,10 @@
           <t>3일</t>
         </is>
       </c>
+      <c r="J56">
+        <f>IF(ROWS($J$2:J56)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J56)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -91047,6 +91265,10 @@
           <t>20,000㎡/일</t>
         </is>
       </c>
+      <c r="J57">
+        <f>IF(ROWS($J$2:J57)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J57)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -91067,6 +91289,10 @@
           <t>20,000㎡/일</t>
         </is>
       </c>
+      <c r="J58">
+        <f>IF(ROWS($J$2:J58)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J58)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -91087,6 +91313,10 @@
           <t>4,900㎡/일</t>
         </is>
       </c>
+      <c r="J59">
+        <f>IF(ROWS($J$2:J59)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J59)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -91107,6 +91337,10 @@
           <t>4,500㎡/일</t>
         </is>
       </c>
+      <c r="J60">
+        <f>IF(ROWS($J$2:J60)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J60)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -91127,6 +91361,10 @@
           <t>4,800㎡/일</t>
         </is>
       </c>
+      <c r="J61">
+        <f>IF(ROWS($J$2:J61)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J61)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -91147,6 +91385,10 @@
           <t>3일/km</t>
         </is>
       </c>
+      <c r="J62">
+        <f>IF(ROWS($J$2:J62)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J62)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -91167,6 +91409,10 @@
           <t>1,900m/일</t>
         </is>
       </c>
+      <c r="J63">
+        <f>IF(ROWS($J$2:J63)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J63)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -91187,6 +91433,10 @@
           <t>1,600m/일</t>
         </is>
       </c>
+      <c r="J64">
+        <f>IF(ROWS($J$2:J64)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J64)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -91207,6 +91457,10 @@
           <t>5일</t>
         </is>
       </c>
+      <c r="J65">
+        <f>IF(ROWS($J$2:J65)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J65)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -91227,6 +91481,10 @@
           <t>600㎥/일</t>
         </is>
       </c>
+      <c r="J66">
+        <f>IF(ROWS($J$2:J66)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J66)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -91247,6 +91505,10 @@
           <t>550㎥/일</t>
         </is>
       </c>
+      <c r="J67">
+        <f>IF(ROWS($J$2:J67)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J67)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -91267,6 +91529,10 @@
           <t>1,900m/일</t>
         </is>
       </c>
+      <c r="J68">
+        <f>IF(ROWS($J$2:J68)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J68)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -91287,6 +91553,10 @@
           <t>1,600m/일</t>
         </is>
       </c>
+      <c r="J69">
+        <f>IF(ROWS($J$2:J69)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J69)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -91307,6 +91577,10 @@
           <t>3일</t>
         </is>
       </c>
+      <c r="J70">
+        <f>IF(ROWS($J$2:J70)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J70)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -91327,6 +91601,10 @@
           <t>300㎥/일</t>
         </is>
       </c>
+      <c r="J71">
+        <f>IF(ROWS($J$2:J71)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J71)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -91347,6 +91625,10 @@
           <t>700㎥/일</t>
         </is>
       </c>
+      <c r="J72">
+        <f>IF(ROWS($J$2:J72)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J72)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -91367,6 +91649,10 @@
           <t>3일</t>
         </is>
       </c>
+      <c r="J73">
+        <f>IF(ROWS($J$2:J73)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J73)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -91387,6 +91673,10 @@
           <t>3일/km</t>
         </is>
       </c>
+      <c r="J74">
+        <f>IF(ROWS($J$2:J74)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J74)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -91407,6 +91697,10 @@
           <t>18일/개소</t>
         </is>
       </c>
+      <c r="J75">
+        <f>IF(ROWS($J$2:J75)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J75)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -91427,6 +91721,10 @@
           <t>10본/일</t>
         </is>
       </c>
+      <c r="J76">
+        <f>IF(ROWS($J$2:J76)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J76)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -91447,6 +91745,10 @@
           <t>10일/1Lot</t>
         </is>
       </c>
+      <c r="J77">
+        <f>IF(ROWS($J$2:J77)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J77)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -91467,6 +91769,10 @@
           <t>7일/1Lot</t>
         </is>
       </c>
+      <c r="J78">
+        <f>IF(ROWS($J$2:J78)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J78)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -91487,6 +91793,10 @@
           <t>20일/개소</t>
         </is>
       </c>
+      <c r="J79">
+        <f>IF(ROWS($J$2:J79)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J79)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -91507,6 +91817,10 @@
           <t>10일</t>
         </is>
       </c>
+      <c r="J80">
+        <f>IF(ROWS($J$2:J80)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J80)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -91527,6 +91841,10 @@
           <t>18일/본</t>
         </is>
       </c>
+      <c r="J81">
+        <f>IF(ROWS($J$2:J81)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J81)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -91547,6 +91865,10 @@
           <t>2본/일</t>
         </is>
       </c>
+      <c r="J82">
+        <f>IF(ROWS($J$2:J82)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J82)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -91567,6 +91889,10 @@
           <t>25일/1경간</t>
         </is>
       </c>
+      <c r="J83">
+        <f>IF(ROWS($J$2:J83)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J83)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -91587,6 +91913,10 @@
           <t>200㎡/일</t>
         </is>
       </c>
+      <c r="J84">
+        <f>IF(ROWS($J$2:J84)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J84)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -91607,6 +91937,10 @@
           <t>8일/경간</t>
         </is>
       </c>
+      <c r="J85">
+        <f>IF(ROWS($J$2:J85)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J85)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -91627,6 +91961,10 @@
           <t>15일/교량</t>
         </is>
       </c>
+      <c r="J86">
+        <f>IF(ROWS($J$2:J86)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J86)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -91647,6 +91985,10 @@
           <t>25일/개소</t>
         </is>
       </c>
+      <c r="J87">
+        <f>IF(ROWS($J$2:J87)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J87)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -91667,6 +92009,10 @@
           <t>25일/개소</t>
         </is>
       </c>
+      <c r="J88">
+        <f>IF(ROWS($J$2:J88)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J88)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -91687,6 +92033,10 @@
           <t>4.3m/일</t>
         </is>
       </c>
+      <c r="J89">
+        <f>IF(ROWS($J$2:J89)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J89)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -91707,6 +92057,10 @@
           <t>4.1m/일</t>
         </is>
       </c>
+      <c r="J90">
+        <f>IF(ROWS($J$2:J90)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J90)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -91727,6 +92081,10 @@
           <t>2.9m/일</t>
         </is>
       </c>
+      <c r="J91">
+        <f>IF(ROWS($J$2:J91)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J91)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -91747,6 +92105,10 @@
           <t>2.6m/일</t>
         </is>
       </c>
+      <c r="J92">
+        <f>IF(ROWS($J$2:J92)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J92)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -91767,6 +92129,10 @@
           <t>7.1m/일</t>
         </is>
       </c>
+      <c r="J93">
+        <f>IF(ROWS($J$2:J93)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J93)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -91787,6 +92153,10 @@
           <t>2.2m/일</t>
         </is>
       </c>
+      <c r="J94">
+        <f>IF(ROWS($J$2:J94)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J94)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -91807,6 +92177,10 @@
           <t>3.6m/일</t>
         </is>
       </c>
+      <c r="J95">
+        <f>IF(ROWS($J$2:J95)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J95)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -91827,6 +92201,10 @@
           <t>2.2m/일</t>
         </is>
       </c>
+      <c r="J96">
+        <f>IF(ROWS($J$2:J96)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J96)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -91847,6 +92225,10 @@
           <t>2.9m/일</t>
         </is>
       </c>
+      <c r="J97">
+        <f>IF(ROWS($J$2:J97)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J97)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -91867,6 +92249,10 @@
           <t>3일/개소</t>
         </is>
       </c>
+      <c r="J98">
+        <f>IF(ROWS($J$2:J98)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J98)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -91887,6 +92273,10 @@
           <t>5일/개소</t>
         </is>
       </c>
+      <c r="J99">
+        <f>IF(ROWS($J$2:J99)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J99)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -91907,6 +92297,10 @@
           <t>50m/일</t>
         </is>
       </c>
+      <c r="J100">
+        <f>IF(ROWS($J$2:J100)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J100)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -91927,6 +92321,10 @@
           <t>25m/3일</t>
         </is>
       </c>
+      <c r="J101">
+        <f>IF(ROWS($J$2:J101)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J101)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -91947,6 +92345,10 @@
           <t>10m/3일</t>
         </is>
       </c>
+      <c r="J102">
+        <f>IF(ROWS($J$2:J102)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J102)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -91967,6 +92369,10 @@
           <t>25일/개소</t>
         </is>
       </c>
+      <c r="J103">
+        <f>IF(ROWS($J$2:J103)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J103)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -91987,6 +92393,10 @@
           <t>300m/일</t>
         </is>
       </c>
+      <c r="J104">
+        <f>IF(ROWS($J$2:J104)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J104)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -92007,6 +92417,10 @@
           <t>130개/일</t>
         </is>
       </c>
+      <c r="J105">
+        <f>IF(ROWS($J$2:J105)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J105)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -92027,6 +92441,10 @@
           <t>19m/일</t>
         </is>
       </c>
+      <c r="J106">
+        <f>IF(ROWS($J$2:J106)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J106)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -92047,6 +92465,10 @@
           <t>5개소/일</t>
         </is>
       </c>
+      <c r="J107">
+        <f>IF(ROWS($J$2:J107)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J107)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -92067,6 +92489,10 @@
           <t>1개소/일</t>
         </is>
       </c>
+      <c r="J108">
+        <f>IF(ROWS($J$2:J108)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J108)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -92087,6 +92513,10 @@
           <t>32m/일</t>
         </is>
       </c>
+      <c r="J109">
+        <f>IF(ROWS($J$2:J109)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J109)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -92107,6 +92537,10 @@
           <t>85㎡/일</t>
         </is>
       </c>
+      <c r="J110">
+        <f>IF(ROWS($J$2:J110)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J110)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -92127,6 +92561,10 @@
           <t>150개/일</t>
         </is>
       </c>
+      <c r="J111">
+        <f>IF(ROWS($J$2:J111)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J111)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -92147,6 +92585,10 @@
           <t>70개/일</t>
         </is>
       </c>
+      <c r="J112">
+        <f>IF(ROWS($J$2:J112)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J112)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -92167,6 +92609,10 @@
           <t>600m/일</t>
         </is>
       </c>
+      <c r="J113">
+        <f>IF(ROWS($J$2:J113)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J113)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -92187,6 +92633,10 @@
           <t>20일/개소</t>
         </is>
       </c>
+      <c r="J114">
+        <f>IF(ROWS($J$2:J114)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J114)-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -92206,6 +92656,10 @@
         <is>
           <t>90㎡/일</t>
         </is>
+      </c>
+      <c r="J115">
+        <f>IF(ROWS($J$2:J115)&lt;=INDEX($H$2:$H$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0)),INDEX($A$2:$A$115,INDEX($G$2:$G$9,MATCH('공기산정(1일작업량)'!$B$26,$F$2:$F$9,0))+ROWS($J$2:J115)-1),"")</f>
+        <v/>
       </c>
     </row>
     <row r="117">

</xml_diff>

<commit_message>
Show appendix-4 original rate text; remove 3m-wide-only asphalt layers from the sewer preset
Claude-Session: https://claude.ai/code/session_01RwMurm2uiMMwxjQxmRaq3G
</commit_message>
<xml_diff>
--- a/공기산정_2026기준.xlsx
+++ b/공기산정_2026기준.xlsx
@@ -3344,7 +3344,7 @@
     <col width="14" customWidth="1" style="92" min="8" max="8"/>
     <col width="14" customWidth="1" style="92" min="9" max="9"/>
     <col width="14" customWidth="1" style="92" min="10" max="10"/>
-    <col width="14" customWidth="1" style="92" min="11" max="11"/>
+    <col width="18" customWidth="1" style="92" min="11" max="11"/>
     <col width="14" customWidth="1" style="92" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -4541,6 +4541,11 @@
           <t>비작업일수</t>
         </is>
       </c>
+      <c r="K28" s="134" t="inlineStr">
+        <is>
+          <t>부록4 원문 표기</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="139">
@@ -4580,6 +4585,10 @@
         <f>IF(ISNUMBER(I29),ROUND(I29-F29,1),"")</f>
         <v/>
       </c>
+      <c r="K29" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A29,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="139">
@@ -4619,6 +4628,10 @@
         <f>IF(ISNUMBER(I30),ROUND(I30-F30,1),"")</f>
         <v/>
       </c>
+      <c r="K30" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A30,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="139">
@@ -4658,6 +4671,10 @@
         <f>IF(ISNUMBER(I31),ROUND(I31-F31,1),"")</f>
         <v/>
       </c>
+      <c r="K31" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A31,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="139">
@@ -4697,6 +4714,10 @@
         <f>IF(ISNUMBER(I32),ROUND(I32-F32,1),"")</f>
         <v/>
       </c>
+      <c r="K32" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A32,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="139">
@@ -4736,6 +4757,10 @@
         <f>IF(ISNUMBER(I33),ROUND(I33-F33,1),"")</f>
         <v/>
       </c>
+      <c r="K33" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A33,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="139">
@@ -4775,6 +4800,10 @@
         <f>IF(ISNUMBER(I34),ROUND(I34-F34,1),"")</f>
         <v/>
       </c>
+      <c r="K34" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A34,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="139">
@@ -4814,6 +4843,10 @@
         <f>IF(ISNUMBER(I35),ROUND(I35-F35,1),"")</f>
         <v/>
       </c>
+      <c r="K35" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A35,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="139">
@@ -4853,6 +4886,10 @@
         <f>IF(ISNUMBER(I36),ROUND(I36-F36,1),"")</f>
         <v/>
       </c>
+      <c r="K36" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A36,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="139">
@@ -4892,6 +4929,10 @@
         <f>IF(ISNUMBER(I37),ROUND(I37-F37,1),"")</f>
         <v/>
       </c>
+      <c r="K37" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A37,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="139">
@@ -4931,6 +4972,10 @@
         <f>IF(ISNUMBER(I38),ROUND(I38-F38,1),"")</f>
         <v/>
       </c>
+      <c r="K38" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A38,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="139">
@@ -4970,6 +5015,10 @@
         <f>IF(ISNUMBER(I39),ROUND(I39-F39,1),"")</f>
         <v/>
       </c>
+      <c r="K39" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A39,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="139">
@@ -5009,6 +5058,10 @@
         <f>IF(ISNUMBER(I40),ROUND(I40-F40,1),"")</f>
         <v/>
       </c>
+      <c r="K40" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A40,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="139">
@@ -5048,6 +5101,10 @@
         <f>IF(ISNUMBER(I41),ROUND(I41-F41,1),"")</f>
         <v/>
       </c>
+      <c r="K41" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A41,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="139">
@@ -5087,6 +5144,10 @@
         <f>IF(ISNUMBER(I42),ROUND(I42-F42,1),"")</f>
         <v/>
       </c>
+      <c r="K42" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A42,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="139">
@@ -5124,6 +5185,10 @@
       </c>
       <c r="J43" s="141">
         <f>IF(ISNUMBER(I43),ROUND(I43-F43,1),"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="141">
+        <f>IFERROR(INDEX('1일작업량(토목)'!$D$2:$D$115,MATCH($A43,'1일작업량(토목)'!$A$2:$A$115,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -92886,7 +92951,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>포장공사&gt;아스팔트포장 2단계-기층 (시공폭 3m 이상, 두께 5-7㎝)</t>
+          <t>굴착부 아스팔트 복구포장 (폭 3m 미만) [1일 작업량 직접 입력]</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -92916,11 +92981,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>포장공사&gt;아스팔트포장 2단계-중간층/표층 (시공폭 3m 이상, 5-7㎝)</t>
-        </is>
-      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>배수공사&gt;배수관-흄관, V.R관 (직경 600mm, 고무링접합)</t>

</xml_diff>